<commit_message>
adds xlsx process & cq
</commit_message>
<xml_diff>
--- a/data/Willy_UneInvention_1895/Willy_UneInvention_1895.xlsx
+++ b/data/Willy_UneInvention_1895/Willy_UneInvention_1895.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mathilde\Desktop\Doctorat - 2025-2028\Pipeline\SFonto\data\Willy_UneInvention_1895\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217069B3-5C8F-454D-82FA-11A014FCD72A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F7A4BD-F8DA-4407-B33C-563499ABD6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="231">
   <si>
     <t>Work</t>
   </si>
@@ -243,9 +243,6 @@
     <t>Classe</t>
   </si>
   <si>
-    <t>E55 Types</t>
-  </si>
-  <si>
     <t>rdf: relation</t>
   </si>
   <si>
@@ -255,9 +252,6 @@
     <t>:Work_Une_Invention</t>
   </si>
   <si>
-    <t>The Invention (work)</t>
-  </si>
-  <si>
     <t xml:space="preserve">dcterms:title </t>
   </si>
   <si>
@@ -345,12 +339,6 @@
     <t>sequences G5 Narrative Event</t>
   </si>
   <si>
-    <t>:Sequence_Fabula</t>
-  </si>
-  <si>
-    <t>:Sequence_Syuzhet</t>
-  </si>
-  <si>
     <t>:type_commercial_institution</t>
   </si>
   <si>
@@ -388,9 +376,6 @@
   </si>
   <si>
     <t>:Time_26_February_1895</t>
-  </si>
-  <si>
-    <t>26th February_1895</t>
   </si>
   <si>
     <t>26th February 1895</t>
@@ -532,54 +517,6 @@
   </si>
   <si>
     <t>La machine ne peut composer de valse en quatre temps</t>
-  </si>
-  <si>
-    <t>:NU01</t>
-  </si>
-  <si>
-    <t>:NU02</t>
-  </si>
-  <si>
-    <t>:NU03</t>
-  </si>
-  <si>
-    <t>:NU04</t>
-  </si>
-  <si>
-    <t>:NU05</t>
-  </si>
-  <si>
-    <t>:NU06</t>
-  </si>
-  <si>
-    <t>:NU07</t>
-  </si>
-  <si>
-    <t>:NU08</t>
-  </si>
-  <si>
-    <t>:NU09</t>
-  </si>
-  <si>
-    <t>:NU10</t>
-  </si>
-  <si>
-    <t>:NU11</t>
-  </si>
-  <si>
-    <t>:NU12</t>
-  </si>
-  <si>
-    <t>:NU13</t>
-  </si>
-  <si>
-    <t>:NU14</t>
-  </si>
-  <si>
-    <t>:NU15</t>
-  </si>
-  <si>
-    <t>:NU16</t>
   </si>
   <si>
     <t>:Function_lack_liquidated</t>
@@ -713,6 +650,93 @@
   </si>
   <si>
     <t>fr</t>
+  </si>
+  <si>
+    <t>novum introduced by</t>
+  </si>
+  <si>
+    <t>:HP4i_is_made_by :Lemice_Terrieux</t>
+  </si>
+  <si>
+    <t>:Feature_first_person_narrator</t>
+  </si>
+  <si>
+    <t>:Sequence_Fabula_Une_Invention</t>
+  </si>
+  <si>
+    <t>:Sequence_Syuzhet_Une_Invention</t>
+  </si>
+  <si>
+    <t>Une Invention (work)</t>
+  </si>
+  <si>
+    <t>:Role_hero</t>
+  </si>
+  <si>
+    <t>H4_Non-Human_Character</t>
+  </si>
+  <si>
+    <t>H5_Personality_Assignment</t>
+  </si>
+  <si>
+    <t>:Automatic_Composer_Intelligence</t>
+  </si>
+  <si>
+    <t>Automatic Composer Intelligence</t>
+  </si>
+  <si>
+    <t>:Positive_Valence</t>
+  </si>
+  <si>
+    <t>:Intellect</t>
+  </si>
+  <si>
+    <t>:NU01_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU02_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU03_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU04_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU05_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU06_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU07_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU08_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU09_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU10_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU11_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU12_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU13_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU14_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU15_Une_Invention</t>
+  </si>
+  <si>
+    <t>:NU16_Une_Invention</t>
   </si>
 </sst>
 </file>
@@ -868,7 +892,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -916,15 +940,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1206,7 +1231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.21875" customWidth="1"/>
@@ -1217,13 +1242,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
     </row>
     <row r="2" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1247,16 +1272,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>73</v>
-      </c>
       <c r="E3" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1267,7 +1292,7 @@
         <v>7</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1311,7 +1336,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1322,7 +1347,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1330,13 +1355,13 @@
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -1344,18 +1369,18 @@
         <v>13</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1366,35 +1391,35 @@
         <v>14</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14" s="5" t="s">
+      <c r="B15" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16" t="s">
-        <v>8</v>
-      </c>
       <c r="E15" s="16" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1402,10 +1427,10 @@
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>222</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1413,9 +1438,20 @@
       <c r="B17" s="16"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="E17" s="22">
+        <v>18</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="20">
         <v>1895</v>
       </c>
     </row>
@@ -1442,15 +1478,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1463,37 +1499,37 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="17" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>102</v>
+        <v>205</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>164</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1503,10 +1539,10 @@
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
       <c r="F4" s="11" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1515,13 +1551,13 @@
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>166</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1530,13 +1566,13 @@
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
       <c r="E6" s="11" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>167</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1545,13 +1581,13 @@
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -1560,13 +1596,13 @@
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>205</v>
+        <v>184</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1575,13 +1611,13 @@
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1590,13 +1626,13 @@
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1605,13 +1641,13 @@
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -1620,13 +1656,13 @@
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>209</v>
+        <v>188</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>173</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1635,13 +1671,13 @@
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>174</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1650,13 +1686,13 @@
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>211</v>
+        <v>190</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1665,13 +1701,13 @@
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>212</v>
+        <v>191</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>176</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1680,13 +1716,13 @@
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
       <c r="E16" s="11" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>177</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1695,13 +1731,13 @@
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>214</v>
+        <v>193</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1710,34 +1746,34 @@
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
       <c r="E18" s="11" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>179</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>103</v>
+        <v>206</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="16" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>164</v>
+        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1747,10 +1783,10 @@
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1759,13 +1795,13 @@
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>166</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1774,13 +1810,13 @@
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
       <c r="E22" s="11" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>167</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1789,13 +1825,13 @@
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1804,13 +1840,13 @@
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
       <c r="E24" s="11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>205</v>
+        <v>184</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1819,13 +1855,13 @@
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1834,13 +1870,13 @@
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
       <c r="E26" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1849,13 +1885,13 @@
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1864,13 +1900,13 @@
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
       <c r="E28" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>209</v>
+        <v>188</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>173</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1879,13 +1915,13 @@
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>174</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1894,13 +1930,13 @@
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
       <c r="E30" s="11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>211</v>
+        <v>190</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1909,13 +1945,13 @@
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>212</v>
+        <v>191</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>176</v>
+        <v>227</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
@@ -1924,13 +1960,13 @@
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
       <c r="E32" s="11" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>177</v>
+        <v>228</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -1939,13 +1975,13 @@
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>214</v>
+        <v>193</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
@@ -1954,34 +1990,34 @@
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
       <c r="E34" s="11" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>179</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="B35" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="B35" s="16" t="s">
-        <v>218</v>
-      </c>
       <c r="C35" s="16" t="s">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1990,13 +2026,13 @@
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
       <c r="E36" s="11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -2005,13 +2041,13 @@
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -2020,13 +2056,13 @@
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -2035,13 +2071,13 @@
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
       <c r="E39" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -2050,13 +2086,13 @@
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
       <c r="E40" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>205</v>
+        <v>184</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>173</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -2065,13 +2101,13 @@
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="F41" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="F41" s="16" t="s">
-        <v>206</v>
-      </c>
       <c r="G41" s="16" t="s">
-        <v>174</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -2080,13 +2116,13 @@
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
       <c r="E42" s="11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -2100,7 +2136,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{370C544A-8303-4EC3-9A95-CF153D35BD7D}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2115,20 +2151,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
     </row>
     <row r="2" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2173,16 +2209,16 @@
         <v>29</v>
       </c>
       <c r="B3" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="16" t="s">
         <v>81</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>83</v>
       </c>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
@@ -2197,26 +2233,28 @@
         <v>29</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="H4" s="6"/>
+      <c r="H4" s="6" t="s">
+        <v>208</v>
+      </c>
       <c r="I4" s="6" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
@@ -2227,7 +2265,7 @@
         <v>29</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
@@ -2243,6 +2281,56 @@
       <c r="J5" s="16"/>
       <c r="K5" s="16"/>
       <c r="L5" s="16"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>213</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2254,28 +2342,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986016D8-19A6-42C1-B729-6B723408289C}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.44140625" customWidth="1"/>
     <col min="2" max="2" width="26.88671875" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="27.77734375" customWidth="1"/>
-    <col min="6" max="6" width="34.77734375" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" style="19" customWidth="1"/>
+    <col min="6" max="6" width="27.77734375" customWidth="1"/>
+    <col min="7" max="7" width="34.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2289,71 +2379,79 @@
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>89</v>
-      </c>
       <c r="D3" s="16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>71</v>
+        <v>203</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
-        <v>71</v>
-      </c>
+      <c r="E4" s="7"/>
       <c r="F4" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D5" s="16"/>
-      <c r="E5" s="16" t="s">
-        <v>71</v>
-      </c>
+      <c r="E5" s="16"/>
       <c r="F5" s="16" t="s">
-        <v>110</v>
+        <v>70</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2373,15 +2471,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2411,10 +2509,10 @@
         <v>41</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>42</v>
@@ -2422,7 +2520,7 @@
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
       <c r="G3" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2430,18 +2528,18 @@
         <v>41</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -2449,18 +2547,18 @@
         <v>41</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -2468,16 +2566,16 @@
         <v>43</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
       <c r="G6" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -2485,16 +2583,16 @@
         <v>41</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2518,14 +2616,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2549,61 +2647,61 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>112</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
@@ -2611,13 +2709,13 @@
     </row>
     <row r="7" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>120</v>
-      </c>
       <c r="C7" s="16" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -2646,16 +2744,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2685,154 +2783,154 @@
     </row>
     <row r="3" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F3" s="16"/>
       <c r="G3" s="16" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2856,14 +2954,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2887,300 +2985,300 @@
     </row>
     <row r="3" spans="1:6" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>164</v>
+        <v>215</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16" t="s">
-        <v>181</v>
+        <v>160</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
       <c r="F4" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>166</v>
+        <v>217</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>167</v>
+        <v>218</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>169</v>
-      </c>
       <c r="C8" s="12" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>173</v>
+        <v>224</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>174</v>
+        <v>225</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>176</v>
+        <v>227</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>177</v>
+        <v>228</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="17" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>179</v>
+        <v>230</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -3212,17 +3310,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -3255,115 +3353,115 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
     </row>
     <row r="5" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>189</v>
+        <v>168</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>194</v>
+        <v>173</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>190</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
       <c r="H6" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>191</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>192</v>
+        <v>171</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -3424,12 +3522,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="2" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -3447,16 +3545,16 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>